<commit_message>
Leads: 2026-10-14 13:32 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://www.provenroof.com/sap/roofers/elgin-il</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>info@provenroof.com</t>
@@ -554,6 +553,122 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Ann Arbor, MI | Brown Chimney</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>brownchimney.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://brownchimney.com/ann-arbor/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Explore Our</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>support@brownchimney.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>248-260-5979</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>heat pump installation Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Service in Ann Arbor</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>dudekheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://dudekheatingandcooling.com/locations/ann-arbor-mi/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@dudekheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(187) 735-9107</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>heat pump installation Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 13:44 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,6 @@
           <t>https://dudekheatingandcooling.com/locations/ann-arbor-mi/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>info@dudekheatingandcooling.com</t>
@@ -669,6 +668,58 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jeff's Plumbing Inc</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>jeffsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.jeffsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>jeff_theplumber@msn.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>76</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>plumber Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 13:45 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -694,13 +694,11 @@
           <t>https://www.jeffsplumbing.com/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>jeff_theplumber@msn.com</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Sacramento CA</t>
@@ -720,6 +718,66 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ICAS Storm Restoration</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>icasstormrestoration.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://icasstormrestoration.com/roofing-central-florida/palm-bay-fl/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bill Smolinsky</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@icasstormrestoration.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(321) 486-8948</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:06 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -783,6 +783,178 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Blue Line Roofing &amp; Exteriors | Central Illinois</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>bluelineroof.net</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.bluelineroof.net/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@bluelineroof.net</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(309) 256-7271</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Peoria IL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roofing contractor Peoria IL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Western Specialty Contractors - Master Craftsmen in Building Envelope Repair</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>westernspecialtycontractors.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://westernspecialtycontractors.com/peoria/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Johnson Vice</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>michaelb@westerngroup.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>309-459-9069</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Peoria IL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roofing contractor Peoria IL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Elite Armour Roofing LLC.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>elitearmourroofing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://elitearmourroofing.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>elitearmourroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(800) 327-4987</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Peoria IL</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofing contractor Peoria IL</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:10 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -804,7 +804,6 @@
           <t>https://www.bluelineroof.net/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>info@bluelineroof.net</t>
@@ -920,7 +919,6 @@
           <t>https://elitearmourroofing.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>elitearmourroofing@gmail.com</t>
@@ -950,6 +948,62 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Drain Cleaning &amp; Clog Removal in Greenville, SC | Teleios Plumbing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>teleiosllc.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.teleiosllc.com/service-areas/greenville-sc-drain-cleaning-clog-removal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@teleiosllc.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(864) 300-4737</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>94</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>drain cleaning service Greenville SC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:13 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -974,7 +974,6 @@
           <t>https://www.teleiosllc.com/service-areas/greenville-sc-drain-cleaning-clog-removal</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>info@teleiosllc.com</t>
@@ -1004,6 +1003,182 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Frisco - Firehouse Roofing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>firehouseroofing.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://firehouseroofing.com/service-areas/frisco/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Founded Roofing</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>admin@keypermarketing.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(214) 888-3152</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofer Frisco TX</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Town &amp; Country Roofing | Frisco TX Roofers</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>townandcountryroofingdfw.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://townandcountryroofingdfw.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@townandcountryroofingdfw.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(972) 377-8188</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>96</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roofer Frisco TX</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Baklava Roofing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>baklavaroofing.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://baklavaroofing.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Allen Finished</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@baklavaroofing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(945) 338-6050</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roofer Frisco TX</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:17 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1089,7 +1089,6 @@
           <t>https://townandcountryroofingdfw.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>info@townandcountryroofingdfw.com</t>
@@ -1179,6 +1178,66 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Premium Metal Roofing in New York – Durable &amp; Stylish</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>rudanroofing.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.rudanroofing.com/new-york</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Rudan Roofing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@rudanroofing.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(416) 299 8586</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>metal roofing contractor New York NY</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:20 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1243,6 +1243,62 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Alpha Home Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>alphahomeroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://alphahomeroofingllc.com/roofing-contractor-in-elizabeth-nj-2/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@alphahomeroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(908) 612-3394</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Elizabeth NJ</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roofing contractor Elizabeth NJ</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:21 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1264,7 +1264,6 @@
           <t>https://alphahomeroofingllc.com/roofing-contractor-in-elizabeth-nj-2/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@alphahomeroofingllc.com</t>
@@ -1294,6 +1293,66 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Star Boy Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>starboyroofing.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://starboyroofing.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Boy Roofing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>roofer6989@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>406-850-7498</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roofing contractor Billings MT</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:23 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1358,6 +1358,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Craftsman Exteriors</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>wisconsincraftsman.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.wisconsincraftsman.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Call For</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>scott@wisconsincraftsman.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(608) 843-5007</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roofer Madison WI</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-14 20:26 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-14.xlsx
+++ b/output/leads_2026-10-14.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1418,6 +1418,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Neptune Air Conditioning, Inc.</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>airconditioninginnyc.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.airconditioninginnyc.com/ac-installation-nyc--new-york-city--ny.html</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@airconditioninginnyc.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>646.863.2132</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>78</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>AC installation New York NY</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>